<commit_message>
feat: add configurable homepage banner carousel
</commit_message>
<xml_diff>
--- a/data/source/glassmartin-products.xlsx
+++ b/data/source/glassmartin-products.xlsx
@@ -9,6 +9,7 @@
     <sheet name="packages" sheetId="4" r:id="rId4"/>
     <sheet name="settings" sheetId="5" r:id="rId5"/>
     <sheet name="promotions" sheetId="6" r:id="rId6"/>
+    <sheet name="banners" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -402,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -460,16 +461,72 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>showroom</v>
+      </c>
+      <c r="B5" t="str">
+        <v>售楼处 / 展厅</v>
+      </c>
+      <c r="C5" t="str">
+        <v>提升来访体验和空间记忆点</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>office</v>
+      </c>
+      <c r="B6" t="str">
+        <v>办公室 / 商务空间</v>
+      </c>
+      <c r="C6" t="str">
+        <v>清爽、克制、适合长时间停留</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>retail</v>
+      </c>
+      <c r="B7" t="str">
+        <v>商场 / 零售门店</v>
+      </c>
+      <c r="C7" t="str">
+        <v>增强品牌识别和停留体验</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>deodorizing</v>
+      </c>
+      <c r="B8" t="str">
+        <v>卫生间 / 除味空间</v>
+      </c>
+      <c r="C8" t="str">
+        <v>强调除味、清洁感和持续扩散</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -558,9 +615,38 @@
         <v>1-3L:参考区间价;4-9L:参考区间价;10L+:参考区间价</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>spa-calm</v>
+      </c>
+      <c r="B4" t="str">
+        <v>静谧会所香</v>
+      </c>
+      <c r="C4" t="str">
+        <v>柔和舒缓，适合会所、SPA 和足浴空间。</v>
+      </c>
+      <c r="D4" t="str">
+        <v>花香 / 木质</v>
+      </c>
+      <c r="E4" t="str">
+        <v>wellness</v>
+      </c>
+      <c r="F4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H4" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I4" t="str">
+        <v>1-3L:参考区间价;4-9L:参考区间价;10L+:参考区间价</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -636,7 +722,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -707,9 +793,32 @@
         <v>gas-501f:2</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>wellness-calm</v>
+      </c>
+      <c r="B4" t="str">
+        <v>会所 SPA 舒缓方案</v>
+      </c>
+      <c r="C4" t="str">
+        <v>wellness</v>
+      </c>
+      <c r="D4" t="str">
+        <v>适合会所、SPA、足浴等停留型空间的香氛方案。</v>
+      </c>
+      <c r="E4" t="str">
+        <v>spa-calm</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4" t="str">
+        <v>gas-501f:1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -796,4 +905,119 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>title</v>
+      </c>
+      <c r="C1" t="str">
+        <v>subtitle</v>
+      </c>
+      <c r="D1" t="str">
+        <v>image</v>
+      </c>
+      <c r="E1" t="str">
+        <v>linkType</v>
+      </c>
+      <c r="F1" t="str">
+        <v>targetId</v>
+      </c>
+      <c r="G1" t="str">
+        <v>sortOrder</v>
+      </c>
+      <c r="H1" t="str">
+        <v>enabled</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>hotel-promo</v>
+      </c>
+      <c r="B2" t="str">
+        <v>酒店空间香氛方案</v>
+      </c>
+      <c r="C2" t="str">
+        <v>为大堂、走廊和客房公共区建立稳定香气记忆</v>
+      </c>
+      <c r="D2" t="str">
+        <v>/images/banners/hotel-lobby.jpg</v>
+      </c>
+      <c r="E2" t="str">
+        <v>scenario</v>
+      </c>
+      <c r="F2" t="str">
+        <v>hotel</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="str">
+        <v>TRUE</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>entertainment-promo</v>
+      </c>
+      <c r="B3" t="str">
+        <v>娱乐商业空间方案</v>
+      </c>
+      <c r="C3" t="str">
+        <v>适合 KTV、酒吧、台球和网咖的高扩散香氛配置</v>
+      </c>
+      <c r="D3" t="str">
+        <v>/images/banners/entertainment.jpg</v>
+      </c>
+      <c r="E3" t="str">
+        <v>scenario</v>
+      </c>
+      <c r="F3" t="str">
+        <v>entertainment</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3" t="str">
+        <v>TRUE</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>wellness-promo</v>
+      </c>
+      <c r="B4" t="str">
+        <v>会所 SPA 舒缓方案</v>
+      </c>
+      <c r="C4" t="str">
+        <v>用柔和香气提升停留感和放松体验</v>
+      </c>
+      <c r="D4" t="str">
+        <v>/images/banners/wellness.jpg</v>
+      </c>
+      <c r="E4" t="str">
+        <v>scenario</v>
+      </c>
+      <c r="F4" t="str">
+        <v>wellness</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+      <c r="H4" t="str">
+        <v>TRUE</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
data: add hotel series scent catalog
</commit_message>
<xml_diff>
--- a/data/source/glassmartin-products.xlsx
+++ b/data/source/glassmartin-products.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -559,19 +559,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>white-tea-hotel</v>
+        <v>gm051801</v>
       </c>
       <c r="B2" t="str">
-        <v>白茶酒店香</v>
+        <v>威斯汀白茶 / Westin White Tea</v>
       </c>
       <c r="C2" t="str">
-        <v>干净、柔和、适合酒店大堂和走廊。</v>
+        <v>酒店系列精油，编号 GM051801。明细气味：白茶、佛手柑、雪松 / White Tea, Bergamot, Cedar。</v>
       </c>
       <c r="D2" t="str">
-        <v>茶香 / 木质</v>
+        <v>茶香花香调 / Tea Floral</v>
       </c>
       <c r="E2" t="str">
-        <v>hotel,office,showroom</v>
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
       </c>
       <c r="F2" t="str">
         <v>TRUE</v>
@@ -583,24 +583,24 @@
         <v>FALSE</v>
       </c>
       <c r="I2" t="str">
-        <v>1-3L:参考区间价;4-9L:参考区间价;10L+:参考区间价</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>night-club-energy</v>
+        <v>gm051802</v>
       </c>
       <c r="B3" t="str">
-        <v>活力娱乐场景香</v>
+        <v>桂花乌龙23 / Osmanthus Oolong 23</v>
       </c>
       <c r="C3" t="str">
-        <v>扩散明显，适合 KTV、酒吧、台球和网咖空间。</v>
+        <v>酒店系列精油，编号 GM051802。明细气味：桂花、乌龙茶、蜜桃 / Osmanthus, Oolong Tea, Peach。</v>
       </c>
       <c r="D3" t="str">
-        <v>果香 / 琥珀</v>
+        <v>茶香花果调 / Tea Floral Fruity</v>
       </c>
       <c r="E3" t="str">
-        <v>entertainment</v>
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
       </c>
       <c r="F3" t="str">
         <v>TRUE</v>
@@ -612,24 +612,24 @@
         <v>FALSE</v>
       </c>
       <c r="I3" t="str">
-        <v>1-3L:参考区间价;4-9L:参考区间价;10L+:参考区间价</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>spa-calm</v>
+        <v>gm051803</v>
       </c>
       <c r="B4" t="str">
-        <v>静谧会所香</v>
+        <v>杜桑的回忆 / Memory of Do Son</v>
       </c>
       <c r="C4" t="str">
-        <v>柔和舒缓，适合会所、SPA 和足浴空间。</v>
+        <v>酒店系列精油，编号 GM051803。明细气味：晚香玉、橙花、麝香 / Tuberose, Orange Blossom, Musk。</v>
       </c>
       <c r="D4" t="str">
-        <v>花香 / 木质</v>
+        <v>白花木质调 / White Floral Woody</v>
       </c>
       <c r="E4" t="str">
-        <v>wellness</v>
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
       </c>
       <c r="F4" t="str">
         <v>TRUE</v>
@@ -641,12 +641,737 @@
         <v>FALSE</v>
       </c>
       <c r="I4" t="str">
-        <v>1-3L:参考区间价;4-9L:参考区间价;10L+:参考区间价</v>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>gm051804</v>
+      </c>
+      <c r="B5" t="str">
+        <v>蓝风铃 / Blue Bell</v>
+      </c>
+      <c r="C5" t="str">
+        <v>酒店系列精油，编号 GM051804。明细气味：风铃草、柿子、白麝香 / Bluebell, Persimmon, White Musk。</v>
+      </c>
+      <c r="D5" t="str">
+        <v>花果清新调 / Fresh Floral Fruity</v>
+      </c>
+      <c r="E5" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F5" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G5" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H5" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>gm051805</v>
+      </c>
+      <c r="B6" t="str">
+        <v>海洋之风 / Ocean Breeze</v>
+      </c>
+      <c r="C6" t="str">
+        <v>酒店系列精油，编号 GM051805。明细气味：海盐、柑橘、海风 / Sea Salt, Citrus, Marine Breeze。</v>
+      </c>
+      <c r="D6" t="str">
+        <v>海洋清新调 / Marine Fresh</v>
+      </c>
+      <c r="E6" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F6" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G6" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H6" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>gm051806</v>
+      </c>
+      <c r="B7" t="str">
+        <v>栀子花 / Gardenia</v>
+      </c>
+      <c r="C7" t="str">
+        <v>酒店系列精油，编号 GM051806。明细气味：栀子花、茉莉、绿叶 / Gardenia, Jasmine, Green Leaves。</v>
+      </c>
+      <c r="D7" t="str">
+        <v>白花调 / White Floral</v>
+      </c>
+      <c r="E7" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H7" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>gm051807</v>
+      </c>
+      <c r="B8" t="str">
+        <v>秋梨苍兰 / Autumn Pear &amp; Freesia</v>
+      </c>
+      <c r="C8" t="str">
+        <v>酒店系列精油，编号 GM051807。明细气味：梨、小苍兰、玫瑰 / Pear, Freesia, Rose。</v>
+      </c>
+      <c r="D8" t="str">
+        <v>果香花香调 / Fruity Floral</v>
+      </c>
+      <c r="E8" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F8" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G8" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H8" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>gm051808</v>
+      </c>
+      <c r="B9" t="str">
+        <v>白茶 / White Tea</v>
+      </c>
+      <c r="C9" t="str">
+        <v>酒店系列精油，编号 GM051808。明细气味：白茶、佛手柑、麝香 / White Tea, Bergamot, Musk。</v>
+      </c>
+      <c r="D9" t="str">
+        <v>茶香木质调 / Tea Woody</v>
+      </c>
+      <c r="E9" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F9" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G9" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H9" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>gm051809</v>
+      </c>
+      <c r="B10" t="str">
+        <v>深定白茶 / Serene White Tea</v>
+      </c>
+      <c r="C10" t="str">
+        <v>酒店系列精油，编号 GM051809。明细气味：白茶、雪松、琥珀 / White Tea, Cedar, Amber。</v>
+      </c>
+      <c r="D10" t="str">
+        <v>茶香木质麝香调 / Tea Woody Musky</v>
+      </c>
+      <c r="E10" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F10" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G10" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H10" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>gm051810</v>
+      </c>
+      <c r="B11" t="str">
+        <v>龙井茶 / Longjing Tea</v>
+      </c>
+      <c r="C11" t="str">
+        <v>酒店系列精油，编号 GM051810。明细气味：龙井茶、竹叶、茉莉 / Longjing Tea, Bamboo Leaf, Jasmine。</v>
+      </c>
+      <c r="D11" t="str">
+        <v>绿茶清香调 / Green Tea Fresh</v>
+      </c>
+      <c r="E11" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F11" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G11" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H11" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>gm051811</v>
+      </c>
+      <c r="B12" t="str">
+        <v>乌木沉香 / Ebony Agarwood</v>
+      </c>
+      <c r="C12" t="str">
+        <v>酒店系列精油，编号 GM051811。明细气味：沉香、乌木、琥珀 / Agarwood, Ebony, Amber。</v>
+      </c>
+      <c r="D12" t="str">
+        <v>木质东方调 / Oriental Woody</v>
+      </c>
+      <c r="E12" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F12" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G12" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H12" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>gm051812</v>
+      </c>
+      <c r="B13" t="str">
+        <v>玫香金漾 / Rosy Golden Glow</v>
+      </c>
+      <c r="C13" t="str">
+        <v>酒店系列精油，编号 GM051812。明细气味：玫瑰、金桂、麝香 / Rose, Golden Osmanthus, Musk。</v>
+      </c>
+      <c r="D13" t="str">
+        <v>花香琥珀调 / Floral Amber</v>
+      </c>
+      <c r="E13" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F13" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G13" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H13" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>gm051813</v>
+      </c>
+      <c r="B14" t="str">
+        <v>白桃乌龙 / White Peach Oolong</v>
+      </c>
+      <c r="C14" t="str">
+        <v>酒店系列精油，编号 GM051813。明细气味：白桃、乌龙茶、茉莉 / White Peach, Oolong Tea, Jasmine。</v>
+      </c>
+      <c r="D14" t="str">
+        <v>茶香果香调 / Tea Fruity</v>
+      </c>
+      <c r="E14" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F14" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G14" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H14" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>gm051814</v>
+      </c>
+      <c r="B15" t="str">
+        <v>大地 / Terre</v>
+      </c>
+      <c r="C15" t="str">
+        <v>酒店系列精油，编号 GM051814。明细气味：葡萄柚、雪松、广藿香 / Grapefruit, Cedar, Patchouli。</v>
+      </c>
+      <c r="D15" t="str">
+        <v>木质柑橘调 / Woody Citrus</v>
+      </c>
+      <c r="E15" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F15" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G15" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H15" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>gm051815</v>
+      </c>
+      <c r="B16" t="str">
+        <v>威尼斯人 / Venetian</v>
+      </c>
+      <c r="C16" t="str">
+        <v>酒店系列精油，编号 GM051815。明细气味：橙花、海风、白麝香 / Neroli, Sea Breeze, White Musk。</v>
+      </c>
+      <c r="D16" t="str">
+        <v>水生花香调 / Aquatic Floral</v>
+      </c>
+      <c r="E16" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F16" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G16" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H16" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>gm051816</v>
+      </c>
+      <c r="B17" t="str">
+        <v>竹露煎茶 / Bamboo Dew Sencha</v>
+      </c>
+      <c r="C17" t="str">
+        <v>酒店系列精油，编号 GM051816。明细气味：煎茶、竹叶、露水 / Sencha, Bamboo Leaf, Dew。</v>
+      </c>
+      <c r="D17" t="str">
+        <v>绿茶清香调 / Green Tea Fresh</v>
+      </c>
+      <c r="E17" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F17" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G17" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H17" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>gm051817</v>
+      </c>
+      <c r="B18" t="str">
+        <v>橙花 / Orange Blossom</v>
+      </c>
+      <c r="C18" t="str">
+        <v>酒店系列精油，编号 GM051817。明细气味：橙花、苦橙叶、茉莉 / Orange Blossom, Petitgrain, Jasmine。</v>
+      </c>
+      <c r="D18" t="str">
+        <v>白花柑橘调 / White Floral Citrus</v>
+      </c>
+      <c r="E18" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F18" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G18" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H18" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>gm051818</v>
+      </c>
+      <c r="B19" t="str">
+        <v>蔚蓝 / Bleu</v>
+      </c>
+      <c r="C19" t="str">
+        <v>酒店系列精油，编号 GM051818。明细气味：柑橘、海风、雪松 / Citrus, Sea Breeze, Cedar。</v>
+      </c>
+      <c r="D19" t="str">
+        <v>海洋木质调 / Marine Woody</v>
+      </c>
+      <c r="E19" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F19" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G19" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H19" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>gm051819</v>
+      </c>
+      <c r="B20" t="str">
+        <v>全季禅茶 / Zen Tea</v>
+      </c>
+      <c r="C20" t="str">
+        <v>酒店系列精油，编号 GM051819。明细气味：香柠檬、绿茶、茉莉 / Bergamot, Green Tea, Jasmine。</v>
+      </c>
+      <c r="D20" t="str">
+        <v>绿叶调 / Green</v>
+      </c>
+      <c r="E20" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F20" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G20" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H20" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>gm051820</v>
+      </c>
+      <c r="B21" t="str">
+        <v>万豪国际 / Marriott</v>
+      </c>
+      <c r="C21" t="str">
+        <v>酒店系列精油，编号 GM051820。明细气味：柑橘、紫罗兰、绿茶 / Citrus, Violet, Green Tea。</v>
+      </c>
+      <c r="D21" t="str">
+        <v>花香调 / Floral</v>
+      </c>
+      <c r="E21" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F21" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G21" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H21" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>gm051821</v>
+      </c>
+      <c r="B22" t="str">
+        <v>喜来登 / Sheraton</v>
+      </c>
+      <c r="C22" t="str">
+        <v>酒店系列精油，编号 GM051821。明细气味：柠檬、罗勒、绿茶 / Lemon, Basil, Green Tea。</v>
+      </c>
+      <c r="D22" t="str">
+        <v>柑橘绿叶调 / Citrus Green</v>
+      </c>
+      <c r="E22" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F22" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G22" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H22" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>gm051822</v>
+      </c>
+      <c r="B23" t="str">
+        <v>新香格里拉 / Shangri-La</v>
+      </c>
+      <c r="C23" t="str">
+        <v>酒店系列精油，编号 GM051822。明细气味：佛手柑、白茶、兰花 / Bergamot, White Tea, Orchid。</v>
+      </c>
+      <c r="D23" t="str">
+        <v>花香调 / Floral</v>
+      </c>
+      <c r="E23" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F23" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G23" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H23" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>gm051823</v>
+      </c>
+      <c r="B24" t="str">
+        <v>威斯汀 / Westin</v>
+      </c>
+      <c r="C24" t="str">
+        <v>酒店系列精油，编号 GM051823。明细气味：茶、青柠、紫苏 / Tea, Lime, Perilla。</v>
+      </c>
+      <c r="D24" t="str">
+        <v>花香绿叶调 / Floral Green</v>
+      </c>
+      <c r="E24" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F24" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G24" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H24" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>gm051824</v>
+      </c>
+      <c r="B25" t="str">
+        <v>希尔顿国际 / Hilton</v>
+      </c>
+      <c r="C25" t="str">
+        <v>酒店系列精油，编号 GM051824。明细气味：西柚、鸢尾、广藿香 / Grapefruit, Iris, Patchouli。</v>
+      </c>
+      <c r="D25" t="str">
+        <v>花香柑橘调 / Floral Citrus</v>
+      </c>
+      <c r="E25" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F25" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G25" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H25" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>gm051825</v>
+      </c>
+      <c r="B26" t="str">
+        <v>洲际酒店 / Intercontinental</v>
+      </c>
+      <c r="C26" t="str">
+        <v>酒店系列精油，编号 GM051825。明细气味：柑橘、姜、橙花 / Citrus, Ginger, Orange Flower。</v>
+      </c>
+      <c r="D26" t="str">
+        <v>绿叶花香调 / Floral Green</v>
+      </c>
+      <c r="E26" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F26" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G26" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H26" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>gm051826</v>
+      </c>
+      <c r="B27" t="str">
+        <v>皇冠假日 / Crowne Plaza</v>
+      </c>
+      <c r="C27" t="str">
+        <v>酒店系列精油，编号 GM051826。明细气味：青柠、雪瓜、玫瑰 / Lime, Melon, Rose。</v>
+      </c>
+      <c r="D27" t="str">
+        <v>花香果香调 / Floral Fruity</v>
+      </c>
+      <c r="E27" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F27" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G27" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H27" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>gm051827</v>
+      </c>
+      <c r="B28" t="str">
+        <v>亚朵酒店 / ATOUR HOTEL</v>
+      </c>
+      <c r="C28" t="str">
+        <v>酒店系列精油，编号 GM051827。明细气味：柑橘、雪松、广藿香 / Citrus, Cedar, Patchouli。</v>
+      </c>
+      <c r="D28" t="str">
+        <v>果香木质调 / Fruity Woody</v>
+      </c>
+      <c r="E28" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F28" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G28" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H28" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>gm051828</v>
+      </c>
+      <c r="B29" t="str">
+        <v>四季酒店 / Four Seasons</v>
+      </c>
+      <c r="C29" t="str">
+        <v>酒店系列精油，编号 GM051828。明细气味：香柠檬、玫瑰木、紫罗兰 / Bergamot, Rosewood, Violet。</v>
+      </c>
+      <c r="D29" t="str">
+        <v>花香调 / Floral</v>
+      </c>
+      <c r="E29" t="str">
+        <v>hotel,entertainment,wellness,showroom,office,retail,deodorizing</v>
+      </c>
+      <c r="F29" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="G29" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H29" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="I29" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -761,7 +1486,7 @@
         <v>适合酒店大堂、走廊等公共区域的基础询价方案。</v>
       </c>
       <c r="E2" t="str">
-        <v>white-tea-hotel</v>
+        <v>gm051801,gm051808</v>
       </c>
       <c r="F2">
         <v>5</v>
@@ -784,7 +1509,7 @@
         <v>适合 KTV、酒吧、台球、网咖等空间的常备询价方案。</v>
       </c>
       <c r="E3" t="str">
-        <v>night-club-energy</v>
+        <v>gm051804,gm051818</v>
       </c>
       <c r="F3">
         <v>6</v>
@@ -807,7 +1532,7 @@
         <v>适合会所、SPA、足浴等停留型空间的香氛方案。</v>
       </c>
       <c r="E4" t="str">
-        <v>spa-calm</v>
+        <v>gm051807,gm051813</v>
       </c>
       <c r="F4">
         <v>3</v>

</xml_diff>